<commit_message>
config updated removed alan and muthu emails aug30,3.56pm
</commit_message>
<xml_diff>
--- a/Birthday wish Bot/Input data for birthdate.xlsx
+++ b/Birthday wish Bot/Input data for birthdate.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="66">
   <si>
     <t>Name</t>
   </si>
@@ -32,9 +32,6 @@
     <t>A.Ruban Jeyapaul</t>
   </si>
   <si>
-    <t>T.Ramesh Raja</t>
-  </si>
-  <si>
     <t>S.Mari Lakshmi</t>
   </si>
   <si>
@@ -119,12 +116,6 @@
     <t>S.Naresh Kumar</t>
   </si>
   <si>
-    <t>Alagappan.M</t>
-  </si>
-  <si>
-    <t>S.Muthukumar</t>
-  </si>
-  <si>
     <t>Lalitha Ram</t>
   </si>
   <si>
@@ -137,9 +128,6 @@
     <t>ruban@titandata.com</t>
   </si>
   <si>
-    <t>ramesh@titandata.com</t>
-  </si>
-  <si>
     <t>lakshmi@titandata.com</t>
   </si>
   <si>
@@ -216,12 +204,6 @@
   </si>
   <si>
     <t>naresh.kumar@e5.ai</t>
-  </si>
-  <si>
-    <t>alagappan.m@e5.ai</t>
-  </si>
-  <si>
-    <t>muthukumar.s@e5.ai</t>
   </si>
   <si>
     <t>lalitha@tiliconveli.com</t>
@@ -283,10 +265,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -616,20 +597,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.42578125" customWidth="1"/>
-    <col min="2" max="2" width="26.7109375" style="5" customWidth="1"/>
+    <col min="2" max="2" width="26.7109375" style="4" customWidth="1"/>
     <col min="3" max="3" width="42.140625" customWidth="1"/>
     <col min="4" max="4" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -637,409 +618,374 @@
       </c>
       <c r="D1" s="1"/>
     </row>
-    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+    <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="7">
+      <c r="B2" s="6">
         <v>44774</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D2" s="3"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="6">
+        <v>44917</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" s="3"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="6">
+        <v>44593</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" s="3"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="6">
+        <v>44781</v>
+      </c>
+      <c r="C5" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="4"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="7">
-        <v>44713</v>
-      </c>
-      <c r="C3" s="10" t="s">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="6">
+        <v>44654</v>
+      </c>
+      <c r="C6" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="4"/>
-      <c r="G3" s="2"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="7">
-        <v>44917</v>
-      </c>
-      <c r="C4" s="10" t="s">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="6">
+        <v>44895</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="4"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="7">
-        <v>44593</v>
-      </c>
-      <c r="C5" s="10" t="s">
+      <c r="D7" s="2"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="6">
+        <v>44739</v>
+      </c>
+      <c r="C8" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D5" s="4"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="7">
-        <v>44781</v>
-      </c>
-      <c r="C6" s="10" t="s">
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="6">
+        <v>44675</v>
+      </c>
+      <c r="C9" s="9" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="7">
-        <v>44654</v>
-      </c>
-      <c r="C7" s="10" t="s">
+      <c r="D9" s="2"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="6">
+        <v>44687</v>
+      </c>
+      <c r="C10" s="9" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="7">
-        <v>44895</v>
-      </c>
-      <c r="C8" s="10" t="s">
+      <c r="D10" s="2"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="6">
+        <v>44873</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="3"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="7">
-        <v>44739</v>
-      </c>
-      <c r="C9" s="10" t="s">
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="6">
+        <v>44631</v>
+      </c>
+      <c r="C12" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="D9" s="3"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="7">
-        <v>44675</v>
-      </c>
-      <c r="C10" s="10" t="s">
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="6">
+        <v>44887</v>
+      </c>
+      <c r="C13" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="3"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="6">
+        <v>44568</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="7">
-        <v>44687</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="D11" s="3"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" s="7">
+      <c r="B15" s="6">
         <v>44873</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C15" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="6">
+        <v>44725</v>
+      </c>
+      <c r="C16" s="9" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B13" s="7">
-        <v>44631</v>
-      </c>
-      <c r="C13" s="10" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="6">
+        <v>44697</v>
+      </c>
+      <c r="C17" s="9" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B14" s="7">
-        <v>44887</v>
-      </c>
-      <c r="C14" s="10" t="s">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="6">
+        <v>44602</v>
+      </c>
+      <c r="C18" s="9" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B15" s="7">
-        <v>44568</v>
-      </c>
-      <c r="C15" s="10" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="6">
+        <v>44607</v>
+      </c>
+      <c r="C19" s="9" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B16" s="7">
-        <v>44873</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" s="7">
-        <v>44725</v>
-      </c>
-      <c r="C17" s="10" t="s">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" s="6">
+        <v>44833</v>
+      </c>
+      <c r="C20" s="9" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="7">
-        <v>44697</v>
-      </c>
-      <c r="C18" s="10" t="s">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" s="6">
+        <v>44748</v>
+      </c>
+      <c r="C21" s="9" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B19" s="7">
-        <v>44602</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B20" s="7">
-        <v>44607</v>
-      </c>
-      <c r="C20" s="10" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B21" s="7">
-        <v>44833</v>
-      </c>
-      <c r="C21" s="10" t="s">
-        <v>57</v>
-      </c>
-    </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="s">
+      <c r="A22" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="7">
-        <v>44748</v>
-      </c>
-      <c r="C22" s="10" t="s">
-        <v>58</v>
+      <c r="B22" s="6">
+        <v>44730</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="7">
-        <v>44730</v>
-      </c>
-      <c r="C23" s="10" t="s">
+      <c r="B23" s="6">
+        <v>44622</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24" s="6">
+        <v>44821</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B25" s="6">
+        <v>44565</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B26" s="6">
+        <v>44907</v>
+      </c>
+      <c r="C26" s="10" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="B24" s="7">
-        <v>44622</v>
-      </c>
-      <c r="C24" s="10" t="s">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B27" s="6">
+        <v>44824</v>
+      </c>
+      <c r="C27" s="9" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="B25" s="7">
-        <v>44821</v>
-      </c>
-      <c r="C25" s="10" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B28" s="6">
+        <v>44633</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" s="6">
+        <v>44733</v>
+      </c>
+      <c r="C29" s="9" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="B26" s="7">
-        <v>44565</v>
-      </c>
-      <c r="C26" s="10" t="s">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B30" s="6">
+        <v>44607</v>
+      </c>
+      <c r="C30" s="9" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="B27" s="7">
-        <v>44907</v>
-      </c>
-      <c r="C27" s="11" t="s">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B31" s="6">
+        <v>44773</v>
+      </c>
+      <c r="C31" s="9" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="B28" s="7">
-        <v>44824</v>
-      </c>
-      <c r="C28" s="10" t="s">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B32" s="6">
+        <v>44568</v>
+      </c>
+      <c r="C32" s="9" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B29" s="7">
-        <v>44633</v>
-      </c>
-      <c r="C29" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B30" s="7">
-        <v>44733</v>
-      </c>
-      <c r="C30" s="10" t="s">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B33" s="6">
+        <v>44731</v>
+      </c>
+      <c r="C33" s="9" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B31" s="7">
-        <v>44607</v>
-      </c>
-      <c r="C31" s="10" t="s">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B34" s="6">
+        <v>44904</v>
+      </c>
+      <c r="C34" s="10" t="s">
         <v>65</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B32" s="7">
-        <v>44773</v>
-      </c>
-      <c r="C32" s="10" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B33" s="7">
-        <v>44627</v>
-      </c>
-      <c r="C33" s="10" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B34" s="7">
-        <v>44880</v>
-      </c>
-      <c r="C34" s="10" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="B35" s="7">
-        <v>44568</v>
-      </c>
-      <c r="C35" s="10" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="B36" s="7">
-        <v>44731</v>
-      </c>
-      <c r="C36" s="10" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B37" s="7">
-        <v>44904</v>
-      </c>
-      <c r="C37" s="11" t="s">
-        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1068,21 +1014,18 @@
     <hyperlink ref="C23" r:id="rId22"/>
     <hyperlink ref="C24" r:id="rId23"/>
     <hyperlink ref="C25" r:id="rId24"/>
-    <hyperlink ref="C26" r:id="rId25"/>
+    <hyperlink ref="C27" r:id="rId25"/>
     <hyperlink ref="C28" r:id="rId26"/>
     <hyperlink ref="C29" r:id="rId27"/>
     <hyperlink ref="C30" r:id="rId28"/>
     <hyperlink ref="C31" r:id="rId29"/>
     <hyperlink ref="C32" r:id="rId30"/>
     <hyperlink ref="C33" r:id="rId31"/>
-    <hyperlink ref="C34" r:id="rId32"/>
-    <hyperlink ref="C35" r:id="rId33"/>
-    <hyperlink ref="C36" r:id="rId34"/>
-    <hyperlink ref="C27" r:id="rId35"/>
-    <hyperlink ref="C37" r:id="rId36"/>
+    <hyperlink ref="C26" r:id="rId32"/>
+    <hyperlink ref="C34" r:id="rId33"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId37"/>
+  <pageSetup orientation="portrait" r:id="rId34"/>
 </worksheet>
 </file>
 

</xml_diff>